<commit_message>
voice: drop the game and BỐC QUẺ lines from the script (33 moments, 55 clips)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0197bQZEhzzFaY44zgCmEqGx
</commit_message>
<xml_diff>
--- a/Bubu_Motion/docs/offline-voice-lines.xlsx
+++ b/Bubu_Motion/docs/offline-voice-lines.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Rules" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lines'!$A$1:$H$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lines'!$A$1:$H$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1372,17 +1372,17 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Trò chơi</t>
+          <t>Học tập</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>game_start</t>
+          <t>focus_start</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>A game round starts</t>
+          <t>HỌC TẬP focus block starts</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1392,35 +1392,31 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Chơi nào!</t>
+          <t>Bắt đầu học thôi! Cố lên bé!</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Bắt đầu thôi!</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>Sẵn sàng chưa? Chơi nào!</t>
-        </is>
-      </c>
+          <t>Tập trung nào!</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
       <c r="H27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Trò chơi</t>
+          <t>Học tập</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>game_win</t>
+          <t>focus_done</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Child wins</t>
+          <t>Focus block finished</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1430,35 +1426,31 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Bé thắng rồi! Giỏi quá!</t>
+          <t>Xong một chặng rồi! Nghỉ chút nhé.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Tuyệt vời!</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>Bé giỏi thật đấy!</t>
-        </is>
-      </c>
+          <t>Giỏi quá, nghỉ tay thôi!</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Trò chơi</t>
+          <t>Học tập</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>game_lose</t>
+          <t>break_over</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Child loses or time is up</t>
+          <t>Break ends</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1468,35 +1460,27 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Tiếc quá! Chơi lại nhé?</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>Suýt nữa thôi!</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>Không sao, lần sau sẽ được!</t>
-        </is>
-      </c>
+          <t>Hết giờ nghỉ rồi, học tiếp nhé!</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr"/>
       <c r="H29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Trò chơi</t>
+          <t>Học tập</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>game_draw</t>
+          <t>focus_voided</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>CỜ CA-RÔ draw</t>
+          <t>Child leaves during a focus block</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1506,7 +1490,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Hòa rồi! Ván nữa nhé?</t>
+          <t>Không sao, lần sau mình học trọn nhé.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr"/>
@@ -1514,571 +1498,135 @@
       <c r="H30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Trò chơi</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>game_bubu_wins</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>CỜ CA-RÔ, Bubu wins</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Nhắc nhở &amp; tin nhắn</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>reminder_due</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>A reminder is due</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Every time (no cap)</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Bé ơi, đến giờ rồi đấy!</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Có lời nhắc cho bé đây!</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr"/>
+      <c r="H31" s="4" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Nhắc nhở &amp; tin nhắn</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>reminder_done</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Child dismisses a reminder</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Fades</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>Bé giỏi lắm!</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Xong rồi, giỏi quá!</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr"/>
+      <c r="H32" s="4" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Nhắc nhở &amp; tin nhắn</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>message_new</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>New message from parents, child nearby</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>Every time</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>Ha, ván này thắng rồi!</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>Ván sau bé gỡ lại nhé!</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr"/>
-      <c r="H31" s="2" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Trò chơi</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>game_record</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>New record</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Every time</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>Kỷ lục mới! Bé siêu quá!</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Phá kỷ lục rồi!</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Trò chơi</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>first_mat_xanh</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>First MẮT XANH game</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>Once ever</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Chạm thật nhanh vào mắt xanh lá nhé!</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr"/>
-      <c r="G33" s="2" t="inlineStr"/>
-      <c r="H33" s="2" t="inlineStr"/>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Bé có tin nhắn của bố mẹ đấy!</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr"/>
+      <c r="G33" s="4" t="inlineStr"/>
+      <c r="H33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Trò chơi</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>first_cham_nhanh</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>First CHẠM NHANH game</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>Once ever</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>Chạm vào chấm trắng trước khi nó biến mất nhé!</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr"/>
-      <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>Trò chơi</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>first_tranh_do</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>First CHẠM NHANH game in TRÁNH ĐỎ mode</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>Once ever</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>Chạm chấm trắng, đừng chạm chấm đỏ nhé!</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr"/>
-      <c r="G35" s="2" t="inlineStr"/>
-      <c r="H35" s="2" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>Trò chơi</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>first_ran</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>First RẮN SĂN MỒI game</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>Once ever</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>Vuốt màn hình để lái rắn nhé!</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="2" t="inlineStr"/>
-      <c r="H36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Trò chơi</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>first_me_cung</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>First MÊ CUNG NGHIÊNG game</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>Once ever</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>Nghiêng nhẹ để lăn bi về đích nhé!</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr"/>
-      <c r="G37" s="2" t="inlineStr"/>
-      <c r="H37" s="2" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Trò chơi</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>first_duong_pho</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>First ĐƯỜNG PHỐ game</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>Once ever</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>Nghiêng trái phải để tránh vật cản nhé!</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr"/>
-      <c r="G38" s="2" t="inlineStr"/>
-      <c r="H38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>Trò chơi</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>first_co_caro</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>First CỜ CA-RÔ game</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>Once ever</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>Ai xếp được ba ô thẳng hàng trước là thắng nhé!</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr"/>
-      <c r="G39" s="2" t="inlineStr"/>
-      <c r="H39" s="2" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>Học tập</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>focus_start</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>HỌC TẬP focus block starts</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>Fades</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>Bắt đầu học thôi! Cố lên bé!</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>Tập trung nào!</t>
-        </is>
-      </c>
-      <c r="G40" s="4" t="inlineStr"/>
-      <c r="H40" s="4" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>Học tập</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>focus_done</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>Focus block finished</t>
-        </is>
-      </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>Every time</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>Xong một chặng rồi! Nghỉ chút nhé.</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>Giỏi quá, nghỉ tay thôi!</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="inlineStr"/>
-      <c r="H41" s="4" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>Học tập</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>break_over</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>Break ends</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>Every time</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>Hết giờ nghỉ rồi, học tiếp nhé!</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr"/>
-      <c r="G42" s="4" t="inlineStr"/>
-      <c r="H42" s="4" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>Học tập</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>focus_voided</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>Child leaves during a focus block</t>
-        </is>
-      </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>Every time</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="inlineStr">
-        <is>
-          <t>Không sao, lần sau mình học trọn nhé.</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr"/>
-      <c r="G43" s="4" t="inlineStr"/>
-      <c r="H43" s="4" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>Nhắc nhở &amp; tin nhắn</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>reminder_due</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>A reminder is due</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>Every time (no cap)</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>Bé ơi, đến giờ rồi đấy!</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>Có lời nhắc cho bé đây!</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr"/>
-      <c r="H44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>Nhắc nhở &amp; tin nhắn</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>reminder_done</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Child dismisses a reminder</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>Fades</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>Bé giỏi lắm!</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>Xong rồi, giỏi quá!</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr"/>
-      <c r="H45" s="2" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Nhắc nhở &amp; tin nhắn</t>
-        </is>
-      </c>
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>message_new</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>New message from parents, child nearby</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Every time</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>Bé có tin nhắn của bố mẹ đấy!</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr"/>
-      <c r="G46" s="2" t="inlineStr"/>
-      <c r="H46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Nhắc nhở &amp; tin nhắn</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>notes_empty</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>GHI CHÚ opened with no notes</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>First 3 times</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
         <is>
           <t>Chưa có ghi chú nào. Bé muốn nhớ gì thì cứ nói nhé!</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr"/>
-      <c r="G47" s="2" t="inlineStr"/>
-      <c r="H47" s="2" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>Bốc quẻ</t>
-        </is>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>fortune</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>BỐC QUẺ opens</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>Once a day</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>Để xem hôm nay bé may mắn thế nào nhé!</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr"/>
-      <c r="G48" s="4" t="inlineStr"/>
-      <c r="H48" s="4" t="inlineStr"/>
+      <c r="F34" s="4" t="inlineStr"/>
+      <c r="G34" s="4" t="inlineStr"/>
+      <c r="H34" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H48"/>
+  <autoFilter ref="A1:H34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2103,7 +1651,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -2200,7 +1747,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="9" t="n"/>
       <c r="B12" s="10" t="n"/>

</xml_diff>

<commit_message>
voice: YÊ instead of HOORAY, record the chosen ElevenLabs voice
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0197bQZEhzzFaY44zgCmEqGx
</commit_message>
<xml_diff>
--- a/Bubu_Motion/docs/offline-voice-lines.xlsx
+++ b/Bubu_Motion/docs/offline-voice-lines.xlsx
@@ -1120,7 +1120,7 @@
       </c>
       <c r="F17" s="17" t="inlineStr">
         <is>
-          <t>HOORAY!!! Bạn giỏi quá</t>
+          <t>YÊ!!! Bạn giỏi quá</t>
         </is>
       </c>
       <c r="G17" s="15" t="n"/>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Recorded in the AI's own voice (Kore by default), so Bubu sounds like one character online and offline.</t>
+          <t>ElevenLabs voice "QUYNH ANH - VOICE COACH" (My Voices), chosen by the user 2026-10-01. No hint line for the thought bubble (user decision).</t>
         </is>
       </c>
     </row>

</xml_diff>